<commit_message>
Corregir nombres de cantón por código DPA y regenerar mapas
- 173 de 221 nombres del Dataset Maestro estaban asignados a otro cantón de la
  misma provincia; los códigos DPA y D1/D2/D3/IBTC no cambian.
- XLSX (datos y Top20) y CSV corregidos; CSV con código DPA de 4 caracteres,
  NOMBRE_CANTON y NOMBRE_PROVINCIA. Reporte de cruce por cantón.
- Mapa interactivo: datos y colores reasignados por código.
- 5 mapas estáticos regenerados desde un único dataset (unión por código DPA);
  02_generar_mapas.py deja de ser un esqueleto.
- Se agregan tabla DPA, GeoJSON con cod_dpa y utilidades de corrección.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TkiSiensucCL54R9dbAAXX
</commit_message>
<xml_diff>
--- a/02_datos/IBTC_Dataset_Maestro_DAT4CCION2026.xlsx
+++ b/02_datos/IBTC_Dataset_Maestro_DAT4CCION2026.xlsx
@@ -1523,7 +1523,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>TAISHA</t>
+          <t>TIWINTZA</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -1588,7 +1588,7 @@
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>PALORA</t>
+          <t>HUAMBOYA</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>ELOY ALFARO</t>
+          <t>MUISNE</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -1718,7 +1718,7 @@
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>SAN JUAN BOSCO</t>
+          <t>PABLO SEXTO</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>TIWINTZA</t>
+          <t>LOGROÑO</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -1848,7 +1848,7 @@
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>PABLO SEXTO</t>
+          <t>TAISHA</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
@@ -1978,7 +1978,7 @@
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>ATACAMES</t>
+          <t>RIOVERDE</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
@@ -2043,7 +2043,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>RIOVERDE</t>
+          <t>ELOY ALFARO</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>TENA</t>
+          <t>ARCHIDONA</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
@@ -2238,7 +2238,7 @@
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>QUININDÉ</t>
+          <t>SAN LORENZO</t>
         </is>
       </c>
       <c r="D15" s="10" t="inlineStr">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>SANTIAGO</t>
+          <t>PALORA</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -2368,7 +2368,7 @@
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>PALANDA</t>
+          <t>YACUAMBI</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>EL TAMBO</t>
+          <t>DÉLEG</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -2498,7 +2498,7 @@
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>SAN LORENZO</t>
+          <t>ATACAMES</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
@@ -2563,7 +2563,7 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>DÉLEG</t>
+          <t>SUSCAL</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -2628,7 +2628,7 @@
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>EL CARMEN</t>
+          <t>PEDERNALES</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
@@ -2693,7 +2693,7 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>PALESTINA</t>
+          <t>PEDRO CARBO</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>SUCRE</t>
+          <t>PAJÁN</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
@@ -2888,7 +2888,7 @@
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>SANTA ISABEL</t>
+          <t>PUCARÁ</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
@@ -3018,7 +3018,7 @@
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>MANTA</t>
+          <t>FLAVIO ALFARO</t>
         </is>
       </c>
       <c r="D27" s="10" t="inlineStr">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>GUAYAQUIL</t>
+          <t>BALZAR</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
@@ -3148,7 +3148,7 @@
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>OÑA</t>
+          <t>SÍGSIG</t>
         </is>
       </c>
       <c r="D29" s="10" t="inlineStr">
@@ -3213,7 +3213,7 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>CELICA</t>
+          <t>GONZANAMÁ</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
@@ -3278,7 +3278,7 @@
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>LOGROÑO</t>
+          <t>SUCÚA</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
@@ -3343,7 +3343,7 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>PENIPE</t>
+          <t>PALLATANGA</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>OLMEDO</t>
+          <t>JARAMIJÓ</t>
         </is>
       </c>
       <c r="D33" s="10" t="inlineStr">
@@ -3473,7 +3473,7 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>PUERTO LÓPEZ</t>
+          <t>SAN VICENTE</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -3538,7 +3538,7 @@
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>PALENQUE</t>
+          <t>VALENCIA</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr">
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>COLIMES</t>
+          <t>ALFREDO BAQUERIZO MORENO (JUJÁN)</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -3798,7 +3798,7 @@
       </c>
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>PIÑAS</t>
+          <t>CHILLA</t>
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr">
@@ -3928,7 +3928,7 @@
       </c>
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>OLMEDO</t>
+          <t>ESPÍNDOLA</t>
         </is>
       </c>
       <c r="D41" s="10" t="inlineStr">
@@ -3993,7 +3993,7 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>SAN FERNANDO</t>
+          <t>OÑA</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
@@ -4188,7 +4188,7 @@
       </c>
       <c r="C45" s="10" t="inlineStr">
         <is>
-          <t>SUCÚA</t>
+          <t>SANTIAGO</t>
         </is>
       </c>
       <c r="D45" s="10" t="inlineStr">
@@ -4253,7 +4253,7 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>GUANO</t>
+          <t>COLTA</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
@@ -4318,7 +4318,7 @@
       </c>
       <c r="C47" s="10" t="inlineStr">
         <is>
-          <t>PEDERNALES</t>
+          <t>JAMA</t>
         </is>
       </c>
       <c r="D47" s="10" t="inlineStr">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>GONZALO PIZARRO</t>
+          <t>CUYABENO</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="C49" s="10" t="inlineStr">
         <is>
-          <t>SAMBORONDÓN</t>
+          <t>EL TRIUNFO</t>
         </is>
       </c>
       <c r="D49" s="10" t="inlineStr">
@@ -4513,7 +4513,7 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>GUAMOTE</t>
+          <t>CHUNCHI</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
@@ -4578,7 +4578,7 @@
       </c>
       <c r="C51" s="10" t="inlineStr">
         <is>
-          <t>PAUTE</t>
+          <t>NABÓN</t>
         </is>
       </c>
       <c r="D51" s="10" t="inlineStr">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>QUINSALOMA</t>
+          <t>PALENQUE</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="C53" s="10" t="inlineStr">
         <is>
-          <t>FRANCISCO DE ORELLANA</t>
+          <t>AGUARICO</t>
         </is>
       </c>
       <c r="D53" s="10" t="inlineStr">
@@ -4838,7 +4838,7 @@
       </c>
       <c r="C55" s="10" t="inlineStr">
         <is>
-          <t>ALAUSÍ</t>
+          <t>GUAMOTE</t>
         </is>
       </c>
       <c r="D55" s="10" t="inlineStr">
@@ -4903,7 +4903,7 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>VINCES</t>
+          <t>PUEBLOVIEJO</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
@@ -4968,7 +4968,7 @@
       </c>
       <c r="C57" s="10" t="inlineStr">
         <is>
-          <t>SIMÓN BOLÍVAR</t>
+          <t>SALITRE</t>
         </is>
       </c>
       <c r="D57" s="10" t="inlineStr">
@@ -5033,7 +5033,7 @@
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>JUNÍN</t>
+          <t>TOSAGUA</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
@@ -5098,7 +5098,7 @@
       </c>
       <c r="C59" s="10" t="inlineStr">
         <is>
-          <t>QUEVEDO</t>
+          <t>VENTANAS</t>
         </is>
       </c>
       <c r="D59" s="10" t="inlineStr">
@@ -5163,7 +5163,7 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>CHINCHIPE</t>
+          <t>NANGARITZA</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
@@ -5293,7 +5293,7 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>TOSAGUA</t>
+          <t>OLMEDO</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
@@ -5358,7 +5358,7 @@
       </c>
       <c r="C63" s="10" t="inlineStr">
         <is>
-          <t>MONTECRISTI</t>
+          <t>CHONE</t>
         </is>
       </c>
       <c r="D63" s="10" t="inlineStr">
@@ -5423,7 +5423,7 @@
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>EL CHACO</t>
+          <t>TENA</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
@@ -5488,7 +5488,7 @@
       </c>
       <c r="C65" s="10" t="inlineStr">
         <is>
-          <t>HUAMBOYA</t>
+          <t>SAN JUAN BOSCO</t>
         </is>
       </c>
       <c r="D65" s="10" t="inlineStr">
@@ -5553,7 +5553,7 @@
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>SANTA LUCÍA</t>
+          <t>SIMÓN BOLÍVAR</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
@@ -5618,7 +5618,7 @@
       </c>
       <c r="C67" s="10" t="inlineStr">
         <is>
-          <t>CHIMBO</t>
+          <t>CHILLANES</t>
         </is>
       </c>
       <c r="D67" s="10" t="inlineStr">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>RIOBAMBA</t>
+          <t>ALAUSÍ</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
@@ -5813,7 +5813,7 @@
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>SAN JACINTO DE YAGUACHI</t>
+          <t>COLIMES</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
@@ -5878,7 +5878,7 @@
       </c>
       <c r="C71" s="10" t="inlineStr">
         <is>
-          <t>PALLATANGA</t>
+          <t>PENIPE</t>
         </is>
       </c>
       <c r="D71" s="10" t="inlineStr">
@@ -5943,7 +5943,7 @@
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>GONZANAMÁ</t>
+          <t>SARAGURO</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C73" s="10" t="inlineStr">
         <is>
-          <t>VALENCIA</t>
+          <t>BABA</t>
         </is>
       </c>
       <c r="D73" s="10" t="inlineStr">
@@ -6073,7 +6073,7 @@
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>VENTANAS</t>
+          <t>VINCES</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
@@ -6203,7 +6203,7 @@
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>GIRÓN</t>
+          <t>GUALACEO</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
@@ -6268,7 +6268,7 @@
       </c>
       <c r="C77" s="10" t="inlineStr">
         <is>
-          <t>PAJÁN</t>
+          <t>24 DE MAYO</t>
         </is>
       </c>
       <c r="D77" s="10" t="inlineStr">
@@ -6333,7 +6333,7 @@
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>ESPÍNDOLA</t>
+          <t>SOZORANGA</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
@@ -6398,7 +6398,7 @@
       </c>
       <c r="C79" s="10" t="inlineStr">
         <is>
-          <t>MUISNE</t>
+          <t>QUININDÉ</t>
         </is>
       </c>
       <c r="D79" s="10" t="inlineStr">
@@ -6528,7 +6528,7 @@
       </c>
       <c r="C81" s="10" t="inlineStr">
         <is>
-          <t>SAQUISILÍ</t>
+          <t>PUJILÍ</t>
         </is>
       </c>
       <c r="D81" s="10" t="inlineStr">
@@ -6593,7 +6593,7 @@
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>GUACHAPALA</t>
+          <t>CAMILO PONCE ENRÍQUEZ</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="C83" s="10" t="inlineStr">
         <is>
-          <t>MILAGRO</t>
+          <t>EL EMPALME</t>
         </is>
       </c>
       <c r="D83" s="10" t="inlineStr">
@@ -6723,7 +6723,7 @@
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>CHONE</t>
+          <t>SANTA ANA</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
@@ -6788,7 +6788,7 @@
       </c>
       <c r="C85" s="10" t="inlineStr">
         <is>
-          <t>JAMA</t>
+          <t>PICHINCHA</t>
         </is>
       </c>
       <c r="D85" s="10" t="inlineStr">
@@ -6853,7 +6853,7 @@
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>24 DE MAYO</t>
+          <t>JUNÍN</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
@@ -6918,7 +6918,7 @@
       </c>
       <c r="C87" s="10" t="inlineStr">
         <is>
-          <t>BIBLIÁN</t>
+          <t>LA TRONCAL</t>
         </is>
       </c>
       <c r="D87" s="10" t="inlineStr">
@@ -6983,7 +6983,7 @@
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>AGUARICO</t>
+          <t>FRANCISCO DE ORELLANA</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
@@ -7048,7 +7048,7 @@
       </c>
       <c r="C89" s="10" t="inlineStr">
         <is>
-          <t>NARANJITO</t>
+          <t>PALESTINA</t>
         </is>
       </c>
       <c r="D89" s="10" t="inlineStr">
@@ -7113,7 +7113,7 @@
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>CENTINELA DEL CÓNDOR</t>
+          <t>PALANDA</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
@@ -7178,7 +7178,7 @@
       </c>
       <c r="C91" s="10" t="inlineStr">
         <is>
-          <t>PORTOVIEJO</t>
+          <t>BOLÍVAR</t>
         </is>
       </c>
       <c r="D91" s="10" t="inlineStr">
@@ -7373,7 +7373,7 @@
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>JARAMIJÓ</t>
+          <t>EL CARMEN</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
@@ -7438,7 +7438,7 @@
       </c>
       <c r="C95" s="10" t="inlineStr">
         <is>
-          <t>MONTALVO</t>
+          <t>BUENA FE</t>
         </is>
       </c>
       <c r="D95" s="10" t="inlineStr">
@@ -7503,7 +7503,7 @@
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>YACUAMBI</t>
+          <t>YANTZAZA</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="C97" s="10" t="inlineStr">
         <is>
-          <t>CAÑAR</t>
+          <t>BIBLIÁN</t>
         </is>
       </c>
       <c r="D97" s="10" t="inlineStr">
@@ -7633,7 +7633,7 @@
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>PLAYAS</t>
+          <t>SANTA LUCÍA</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
@@ -7698,7 +7698,7 @@
       </c>
       <c r="C99" s="10" t="inlineStr">
         <is>
-          <t>CEVALLOS</t>
+          <t>SANTIAGO DE PÍLLARO</t>
         </is>
       </c>
       <c r="D99" s="10" t="inlineStr">
@@ -7828,7 +7828,7 @@
       </c>
       <c r="C101" s="10" t="inlineStr">
         <is>
-          <t>BOLÍVAR</t>
+          <t>SUCRE</t>
         </is>
       </c>
       <c r="D101" s="10" t="inlineStr">
@@ -7893,7 +7893,7 @@
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>YANTZAZA</t>
+          <t>EL PANGUI</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
@@ -8023,7 +8023,7 @@
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>SUCUMBÍOS</t>
+          <t>PUTUMAYO</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
@@ -8153,7 +8153,7 @@
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>BUENA FE</t>
+          <t>MOCACHE</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
@@ -8283,7 +8283,7 @@
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>PUCARÁ</t>
+          <t>SAN FERNANDO</t>
         </is>
       </c>
       <c r="D108" s="4" t="inlineStr">
@@ -8348,7 +8348,7 @@
       </c>
       <c r="C109" s="10" t="inlineStr">
         <is>
-          <t>EL PAN</t>
+          <t>GUACHAPALA</t>
         </is>
       </c>
       <c r="D109" s="10" t="inlineStr">
@@ -8413,7 +8413,7 @@
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>CAMILO PONCE ENRÍQUEZ</t>
+          <t>SANTA ISABEL</t>
         </is>
       </c>
       <c r="D110" s="4" t="inlineStr">
@@ -8478,7 +8478,7 @@
       </c>
       <c r="C111" s="10" t="inlineStr">
         <is>
-          <t>ALFREDO BAQUERIZO MORENO (JUJÁN)</t>
+          <t>PLAYAS</t>
         </is>
       </c>
       <c r="D111" s="10" t="inlineStr">
@@ -8543,7 +8543,7 @@
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>BABA</t>
+          <t>MONTALVO</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
@@ -8608,7 +8608,7 @@
       </c>
       <c r="C113" s="10" t="inlineStr">
         <is>
-          <t>ARENILLAS</t>
+          <t>EL GUABO</t>
         </is>
       </c>
       <c r="D113" s="10" t="inlineStr">
@@ -8673,7 +8673,7 @@
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>PICHINCHA</t>
+          <t>PUERTO LÓPEZ</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
@@ -8738,7 +8738,7 @@
       </c>
       <c r="C115" s="10" t="inlineStr">
         <is>
-          <t>BALZAR</t>
+          <t>DURÁN</t>
         </is>
       </c>
       <c r="D115" s="10" t="inlineStr">
@@ -8803,7 +8803,7 @@
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>PUJILÍ</t>
+          <t>LA MANÁ</t>
         </is>
       </c>
       <c r="D116" s="4" t="inlineStr">
@@ -8998,7 +8998,7 @@
       </c>
       <c r="C119" s="10" t="inlineStr">
         <is>
-          <t>CHAGUARPAMBA</t>
+          <t>OLMEDO</t>
         </is>
       </c>
       <c r="D119" s="10" t="inlineStr">
@@ -9063,7 +9063,7 @@
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>SANTA ANA</t>
+          <t>MONTECRISTI</t>
         </is>
       </c>
       <c r="D120" s="4" t="inlineStr">
@@ -9128,7 +9128,7 @@
       </c>
       <c r="C121" s="10" t="inlineStr">
         <is>
-          <t>PALTAS</t>
+          <t>CHAGUARPAMBA</t>
         </is>
       </c>
       <c r="D121" s="10" t="inlineStr">
@@ -9323,7 +9323,7 @@
       </c>
       <c r="C124" s="4" t="inlineStr">
         <is>
-          <t>EL PANGUI</t>
+          <t>CENTINELA DEL CÓNDOR</t>
         </is>
       </c>
       <c r="D124" s="4" t="inlineStr">
@@ -9388,7 +9388,7 @@
       </c>
       <c r="C125" s="10" t="inlineStr">
         <is>
-          <t>ZAMORA</t>
+          <t>CHINCHIPE</t>
         </is>
       </c>
       <c r="D125" s="10" t="inlineStr">
@@ -9518,7 +9518,7 @@
       </c>
       <c r="C127" s="10" t="inlineStr">
         <is>
-          <t>EL EMPALME</t>
+          <t>BALAO</t>
         </is>
       </c>
       <c r="D127" s="10" t="inlineStr">
@@ -9583,7 +9583,7 @@
       </c>
       <c r="C128" s="4" t="inlineStr">
         <is>
-          <t>EL TRIUNFO</t>
+          <t>NARANJITO</t>
         </is>
       </c>
       <c r="D128" s="4" t="inlineStr">
@@ -9713,7 +9713,7 @@
       </c>
       <c r="C130" s="4" t="inlineStr">
         <is>
-          <t>SÍGSIG</t>
+          <t>PAUTE</t>
         </is>
       </c>
       <c r="D130" s="4" t="inlineStr">
@@ -9778,7 +9778,7 @@
       </c>
       <c r="C131" s="10" t="inlineStr">
         <is>
-          <t>MOCACHE</t>
+          <t>QUINSALOMA</t>
         </is>
       </c>
       <c r="D131" s="10" t="inlineStr">
@@ -9843,7 +9843,7 @@
       </c>
       <c r="C132" s="4" t="inlineStr">
         <is>
-          <t>ARCHIDONA</t>
+          <t>CARLOS JULIO AROSEMENA TOLA</t>
         </is>
       </c>
       <c r="D132" s="4" t="inlineStr">
@@ -9908,7 +9908,7 @@
       </c>
       <c r="C133" s="10" t="inlineStr">
         <is>
-          <t>NABÓN</t>
+          <t>CHORDELEG</t>
         </is>
       </c>
       <c r="D133" s="10" t="inlineStr">
@@ -10038,7 +10038,7 @@
       </c>
       <c r="C135" s="10" t="inlineStr">
         <is>
-          <t>SALCEDO</t>
+          <t>PANGUA</t>
         </is>
       </c>
       <c r="D135" s="10" t="inlineStr">
@@ -10103,7 +10103,7 @@
       </c>
       <c r="C136" s="4" t="inlineStr">
         <is>
-          <t>LOJA</t>
+          <t>CATAMAYO</t>
         </is>
       </c>
       <c r="D136" s="4" t="inlineStr">
@@ -10168,7 +10168,7 @@
       </c>
       <c r="C137" s="10" t="inlineStr">
         <is>
-          <t>DURÁN</t>
+          <t>SAN JACINTO DE YAGUACHI</t>
         </is>
       </c>
       <c r="D137" s="10" t="inlineStr">
@@ -10233,7 +10233,7 @@
       </c>
       <c r="C138" s="4" t="inlineStr">
         <is>
-          <t>PUEBLOVIEJO</t>
+          <t>QUEVEDO</t>
         </is>
       </c>
       <c r="D138" s="4" t="inlineStr">
@@ -10298,7 +10298,7 @@
       </c>
       <c r="C139" s="10" t="inlineStr">
         <is>
-          <t>PATATE</t>
+          <t>QUERO</t>
         </is>
       </c>
       <c r="D139" s="10" t="inlineStr">
@@ -10428,7 +10428,7 @@
       </c>
       <c r="C141" s="10" t="inlineStr">
         <is>
-          <t>PUTUMAYO</t>
+          <t>SHUSHUFINDI</t>
         </is>
       </c>
       <c r="D141" s="10" t="inlineStr">
@@ -10558,7 +10558,7 @@
       </c>
       <c r="C143" s="10" t="inlineStr">
         <is>
-          <t>LA MANÁ</t>
+          <t>SAQUISILÍ</t>
         </is>
       </c>
       <c r="D143" s="10" t="inlineStr">
@@ -10623,7 +10623,7 @@
       </c>
       <c r="C144" s="4" t="inlineStr">
         <is>
-          <t>SALITRE</t>
+          <t>MILAGRO</t>
         </is>
       </c>
       <c r="D144" s="4" t="inlineStr">
@@ -10688,7 +10688,7 @@
       </c>
       <c r="C145" s="10" t="inlineStr">
         <is>
-          <t>MACARÁ</t>
+          <t>PALTAS</t>
         </is>
       </c>
       <c r="D145" s="10" t="inlineStr">
@@ -10753,7 +10753,7 @@
       </c>
       <c r="C146" s="4" t="inlineStr">
         <is>
-          <t>SUSCAL</t>
+          <t>CAÑAR</t>
         </is>
       </c>
       <c r="D146" s="4" t="inlineStr">
@@ -10818,7 +10818,7 @@
       </c>
       <c r="C147" s="10" t="inlineStr">
         <is>
-          <t>SANTA ELENA</t>
+          <t>LA LIBERTAD</t>
         </is>
       </c>
       <c r="D147" s="10" t="inlineStr">
@@ -10883,7 +10883,7 @@
       </c>
       <c r="C148" s="4" t="inlineStr">
         <is>
-          <t>BALSAS</t>
+          <t>LAS LAJAS</t>
         </is>
       </c>
       <c r="D148" s="4" t="inlineStr">
@@ -10948,7 +10948,7 @@
       </c>
       <c r="C149" s="10" t="inlineStr">
         <is>
-          <t>ZAPOTILLO</t>
+          <t>CALVAS</t>
         </is>
       </c>
       <c r="D149" s="10" t="inlineStr">
@@ -11013,7 +11013,7 @@
       </c>
       <c r="C150" s="4" t="inlineStr">
         <is>
-          <t>CHORDELEG</t>
+          <t>EL PAN</t>
         </is>
       </c>
       <c r="D150" s="4" t="inlineStr">
@@ -11078,7 +11078,7 @@
       </c>
       <c r="C151" s="10" t="inlineStr">
         <is>
-          <t>CALVAS</t>
+          <t>MACARÁ</t>
         </is>
       </c>
       <c r="D151" s="10" t="inlineStr">
@@ -11143,7 +11143,7 @@
       </c>
       <c r="C152" s="4" t="inlineStr">
         <is>
-          <t>SALINAS</t>
+          <t>SANTA ELENA</t>
         </is>
       </c>
       <c r="D152" s="4" t="inlineStr">
@@ -11208,7 +11208,7 @@
       </c>
       <c r="C153" s="10" t="inlineStr">
         <is>
-          <t>GUALACEO</t>
+          <t>GIRÓN</t>
         </is>
       </c>
       <c r="D153" s="10" t="inlineStr">
@@ -11338,7 +11338,7 @@
       </c>
       <c r="C155" s="10" t="inlineStr">
         <is>
-          <t>SAN MIGUEL</t>
+          <t>CHIMBO</t>
         </is>
       </c>
       <c r="D155" s="10" t="inlineStr">
@@ -11403,7 +11403,7 @@
       </c>
       <c r="C156" s="4" t="inlineStr">
         <is>
-          <t>SOZORANGA</t>
+          <t>ZAPOTILLO</t>
         </is>
       </c>
       <c r="D156" s="4" t="inlineStr">
@@ -11468,7 +11468,7 @@
       </c>
       <c r="C157" s="10" t="inlineStr">
         <is>
-          <t>DISTRITO METROPOLITANO DE QUITO</t>
+          <t>PEDRO MONCAYO</t>
         </is>
       </c>
       <c r="D157" s="10" t="inlineStr">
@@ -11533,7 +11533,7 @@
       </c>
       <c r="C158" s="4" t="inlineStr">
         <is>
-          <t>CHILLANES</t>
+          <t>ECHEANDÍA</t>
         </is>
       </c>
       <c r="D158" s="4" t="inlineStr">
@@ -11598,7 +11598,7 @@
       </c>
       <c r="C159" s="10" t="inlineStr">
         <is>
-          <t>ECHEANDÍA</t>
+          <t>SAN MIGUEL</t>
         </is>
       </c>
       <c r="D159" s="10" t="inlineStr">
@@ -11663,7 +11663,7 @@
       </c>
       <c r="C160" s="4" t="inlineStr">
         <is>
-          <t>SARAGURO</t>
+          <t>CELICA</t>
         </is>
       </c>
       <c r="D160" s="4" t="inlineStr">
@@ -11793,7 +11793,7 @@
       </c>
       <c r="C162" s="4" t="inlineStr">
         <is>
-          <t>CHILLA</t>
+          <t>MARCABELÍ</t>
         </is>
       </c>
       <c r="D162" s="4" t="inlineStr">
@@ -11858,7 +11858,7 @@
       </c>
       <c r="C163" s="10" t="inlineStr">
         <is>
-          <t>LA LIBERTAD</t>
+          <t>SALINAS</t>
         </is>
       </c>
       <c r="D163" s="10" t="inlineStr">
@@ -11923,7 +11923,7 @@
       </c>
       <c r="C164" s="4" t="inlineStr">
         <is>
-          <t>LA TRONCAL</t>
+          <t>EL TAMBO</t>
         </is>
       </c>
       <c r="D164" s="4" t="inlineStr">
@@ -12053,7 +12053,7 @@
       </c>
       <c r="C166" s="4" t="inlineStr">
         <is>
-          <t>SAN VICENTE</t>
+          <t>ROCAFUERTE</t>
         </is>
       </c>
       <c r="D166" s="4" t="inlineStr">
@@ -12118,7 +12118,7 @@
       </c>
       <c r="C167" s="10" t="inlineStr">
         <is>
-          <t>CUYABENO</t>
+          <t>GONZALO PIZARRO</t>
         </is>
       </c>
       <c r="D167" s="10" t="inlineStr">
@@ -12183,7 +12183,7 @@
       </c>
       <c r="C168" s="4" t="inlineStr">
         <is>
-          <t>MIRA</t>
+          <t>BOLÍVAR</t>
         </is>
       </c>
       <c r="D168" s="4" t="inlineStr">
@@ -12313,7 +12313,7 @@
       </c>
       <c r="C170" s="4" t="inlineStr">
         <is>
-          <t>BAÑOS DE AGUA SANTA</t>
+          <t>PATATE</t>
         </is>
       </c>
       <c r="D170" s="4" t="inlineStr">
@@ -12378,7 +12378,7 @@
       </c>
       <c r="C171" s="10" t="inlineStr">
         <is>
-          <t>ZARUMA</t>
+          <t>ATAHUALPA</t>
         </is>
       </c>
       <c r="D171" s="10" t="inlineStr">
@@ -12443,7 +12443,7 @@
       </c>
       <c r="C172" s="4" t="inlineStr">
         <is>
-          <t>CHUNCHI</t>
+          <t>GUANO</t>
         </is>
       </c>
       <c r="D172" s="4" t="inlineStr">
@@ -12508,7 +12508,7 @@
       </c>
       <c r="C173" s="10" t="inlineStr">
         <is>
-          <t>LAS LAJAS</t>
+          <t>SANTA ROSA</t>
         </is>
       </c>
       <c r="D173" s="10" t="inlineStr">
@@ -12573,7 +12573,7 @@
       </c>
       <c r="C174" s="4" t="inlineStr">
         <is>
-          <t>PANGUA</t>
+          <t>SALCEDO</t>
         </is>
       </c>
       <c r="D174" s="4" t="inlineStr">
@@ -12638,7 +12638,7 @@
       </c>
       <c r="C175" s="10" t="inlineStr">
         <is>
-          <t>SANTA ROSA</t>
+          <t>ARENILLAS</t>
         </is>
       </c>
       <c r="D175" s="10" t="inlineStr">
@@ -12703,7 +12703,7 @@
       </c>
       <c r="C176" s="4" t="inlineStr">
         <is>
-          <t>FLAVIO ALFARO</t>
+          <t>PORTOVIEJO</t>
         </is>
       </c>
       <c r="D176" s="4" t="inlineStr">
@@ -12768,7 +12768,7 @@
       </c>
       <c r="C177" s="10" t="inlineStr">
         <is>
-          <t>EL GUABO</t>
+          <t>HUAQUILLAS</t>
         </is>
       </c>
       <c r="D177" s="10" t="inlineStr">
@@ -12963,7 +12963,7 @@
       </c>
       <c r="C180" s="4" t="inlineStr">
         <is>
-          <t>PORTOVELO</t>
+          <t>PASAJE</t>
         </is>
       </c>
       <c r="D180" s="4" t="inlineStr">
@@ -13028,7 +13028,7 @@
       </c>
       <c r="C181" s="10" t="inlineStr">
         <is>
-          <t>COLTA</t>
+          <t>CHAMBO</t>
         </is>
       </c>
       <c r="D181" s="10" t="inlineStr">
@@ -13158,7 +13158,7 @@
       </c>
       <c r="C183" s="10" t="inlineStr">
         <is>
-          <t>NANGARITZA</t>
+          <t>ZAMORA</t>
         </is>
       </c>
       <c r="D183" s="10" t="inlineStr">
@@ -13288,7 +13288,7 @@
       </c>
       <c r="C185" s="10" t="inlineStr">
         <is>
-          <t>BOLÍVAR</t>
+          <t>MIRA</t>
         </is>
       </c>
       <c r="D185" s="10" t="inlineStr">
@@ -13418,7 +13418,7 @@
       </c>
       <c r="C187" s="10" t="inlineStr">
         <is>
-          <t>QUERO</t>
+          <t>SAN PEDRO DE PELILEO</t>
         </is>
       </c>
       <c r="D187" s="10" t="inlineStr">
@@ -13483,7 +13483,7 @@
       </c>
       <c r="C188" s="4" t="inlineStr">
         <is>
-          <t>MARCABELÍ</t>
+          <t>ZARUMA</t>
         </is>
       </c>
       <c r="D188" s="4" t="inlineStr">
@@ -13548,7 +13548,7 @@
       </c>
       <c r="C189" s="10" t="inlineStr">
         <is>
-          <t>ROCAFUERTE</t>
+          <t>MANTA</t>
         </is>
       </c>
       <c r="D189" s="10" t="inlineStr">
@@ -13613,7 +13613,7 @@
       </c>
       <c r="C190" s="4" t="inlineStr">
         <is>
-          <t>BALAO</t>
+          <t>GUAYAQUIL</t>
         </is>
       </c>
       <c r="D190" s="4" t="inlineStr">
@@ -13678,7 +13678,7 @@
       </c>
       <c r="C191" s="10" t="inlineStr">
         <is>
-          <t>CARLOS JULIO AROSEMENA TOLA</t>
+          <t>EL CHACO</t>
         </is>
       </c>
       <c r="D191" s="10" t="inlineStr">
@@ -13743,7 +13743,7 @@
       </c>
       <c r="C192" s="4" t="inlineStr">
         <is>
-          <t>ANTONIO ANTE</t>
+          <t>OTAVALO</t>
         </is>
       </c>
       <c r="D192" s="4" t="inlineStr">
@@ -13808,7 +13808,7 @@
       </c>
       <c r="C193" s="10" t="inlineStr">
         <is>
-          <t>PEDRO MONCAYO</t>
+          <t>CAYAMBE</t>
         </is>
       </c>
       <c r="D193" s="10" t="inlineStr">
@@ -13938,7 +13938,7 @@
       </c>
       <c r="C195" s="10" t="inlineStr">
         <is>
-          <t>MOCHA</t>
+          <t>TISALEO</t>
         </is>
       </c>
       <c r="D195" s="10" t="inlineStr">
@@ -14068,7 +14068,7 @@
       </c>
       <c r="C197" s="10" t="inlineStr">
         <is>
-          <t>ATAHUALPA</t>
+          <t>PORTOVELO</t>
         </is>
       </c>
       <c r="D197" s="10" t="inlineStr">
@@ -14263,7 +14263,7 @@
       </c>
       <c r="C200" s="4" t="inlineStr">
         <is>
-          <t>RUMIÑAHUI</t>
+          <t>MEJÍA</t>
         </is>
       </c>
       <c r="D200" s="4" t="inlineStr">
@@ -14328,7 +14328,7 @@
       </c>
       <c r="C201" s="10" t="inlineStr">
         <is>
-          <t>HUAQUILLAS</t>
+          <t>PIÑAS</t>
         </is>
       </c>
       <c r="D201" s="10" t="inlineStr">
@@ -14393,7 +14393,7 @@
       </c>
       <c r="C202" s="4" t="inlineStr">
         <is>
-          <t>MONTÚFAR</t>
+          <t>ESPEJO</t>
         </is>
       </c>
       <c r="D202" s="4" t="inlineStr">
@@ -14458,7 +14458,7 @@
       </c>
       <c r="C203" s="10" t="inlineStr">
         <is>
-          <t>TULCÁN</t>
+          <t>MONTÚFAR</t>
         </is>
       </c>
       <c r="D203" s="10" t="inlineStr">
@@ -14588,7 +14588,7 @@
       </c>
       <c r="C205" s="10" t="inlineStr">
         <is>
-          <t>TISALEO</t>
+          <t>AMBATO</t>
         </is>
       </c>
       <c r="D205" s="10" t="inlineStr">
@@ -14653,7 +14653,7 @@
       </c>
       <c r="C206" s="4" t="inlineStr">
         <is>
-          <t>PASAJE</t>
+          <t>BALSAS</t>
         </is>
       </c>
       <c r="D206" s="4" t="inlineStr">
@@ -14783,7 +14783,7 @@
       </c>
       <c r="C208" s="4" t="inlineStr">
         <is>
-          <t>ESPEJO</t>
+          <t>TULCÁN</t>
         </is>
       </c>
       <c r="D208" s="4" t="inlineStr">
@@ -14848,7 +14848,7 @@
       </c>
       <c r="C209" s="10" t="inlineStr">
         <is>
-          <t>SAN PEDRO DE PELILEO</t>
+          <t>CEVALLOS</t>
         </is>
       </c>
       <c r="D209" s="10" t="inlineStr">
@@ -14913,7 +14913,7 @@
       </c>
       <c r="C210" s="4" t="inlineStr">
         <is>
-          <t>SHUSHUFINDI</t>
+          <t>SUCUMBÍOS</t>
         </is>
       </c>
       <c r="D210" s="4" t="inlineStr">
@@ -15043,7 +15043,7 @@
       </c>
       <c r="C212" s="4" t="inlineStr">
         <is>
-          <t>ISABELA</t>
+          <t>SANTA CRUZ</t>
         </is>
       </c>
       <c r="D212" s="4" t="inlineStr">
@@ -15108,7 +15108,7 @@
       </c>
       <c r="C213" s="10" t="inlineStr">
         <is>
-          <t>CATAMAYO</t>
+          <t>LOJA</t>
         </is>
       </c>
       <c r="D213" s="10" t="inlineStr">
@@ -15238,7 +15238,7 @@
       </c>
       <c r="C215" s="10" t="inlineStr">
         <is>
-          <t>CHAMBO</t>
+          <t>RIOBAMBA</t>
         </is>
       </c>
       <c r="D215" s="10" t="inlineStr">
@@ -15303,7 +15303,7 @@
       </c>
       <c r="C216" s="4" t="inlineStr">
         <is>
-          <t>SANTA CRUZ</t>
+          <t>ISABELA</t>
         </is>
       </c>
       <c r="D216" s="4" t="inlineStr">
@@ -15368,7 +15368,7 @@
       </c>
       <c r="C217" s="10" t="inlineStr">
         <is>
-          <t>OTAVALO</t>
+          <t>ANTONIO ANTE</t>
         </is>
       </c>
       <c r="D217" s="10" t="inlineStr">
@@ -15433,7 +15433,7 @@
       </c>
       <c r="C218" s="4" t="inlineStr">
         <is>
-          <t>SANTIAGO DE PÍLLARO</t>
+          <t>MOCHA</t>
         </is>
       </c>
       <c r="D218" s="4" t="inlineStr">
@@ -15498,7 +15498,7 @@
       </c>
       <c r="C219" s="10" t="inlineStr">
         <is>
-          <t>AMBATO</t>
+          <t>BAÑOS DE AGUA SANTA</t>
         </is>
       </c>
       <c r="D219" s="10" t="inlineStr">
@@ -15563,7 +15563,7 @@
       </c>
       <c r="C220" s="4" t="inlineStr">
         <is>
-          <t>PEDRO CARBO</t>
+          <t>SAMBORONDÓN</t>
         </is>
       </c>
       <c r="D220" s="4" t="inlineStr">
@@ -15758,7 +15758,7 @@
       </c>
       <c r="C223" s="10" t="inlineStr">
         <is>
-          <t>CAYAMBE</t>
+          <t>DISTRITO METROPOLITANO DE QUITO</t>
         </is>
       </c>
       <c r="D223" s="10" t="inlineStr">
@@ -15823,7 +15823,7 @@
       </c>
       <c r="C224" s="4" t="inlineStr">
         <is>
-          <t>MEJÍA</t>
+          <t>RUMIÑAHUI</t>
         </is>
       </c>
       <c r="D224" s="4" t="inlineStr">
@@ -16126,7 +16126,7 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>TAISHA</t>
+          <t>TIWINTZA</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
@@ -16158,7 +16158,7 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>PALORA</t>
+          <t>HUAMBOYA</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
@@ -16190,7 +16190,7 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>ELOY ALFARO</t>
+          <t>MUISNE</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
@@ -16222,7 +16222,7 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>SAN JUAN BOSCO</t>
+          <t>PABLO SEXTO</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
@@ -16254,7 +16254,7 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>TIWINTZA</t>
+          <t>LOGROÑO</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
@@ -16286,7 +16286,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>PABLO SEXTO</t>
+          <t>TAISHA</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -16350,7 +16350,7 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>ATACAMES</t>
+          <t>RIOVERDE</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
@@ -16382,7 +16382,7 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>RIOVERDE</t>
+          <t>ELOY ALFARO</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
@@ -16414,7 +16414,7 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>TENA</t>
+          <t>ARCHIDONA</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
@@ -16478,7 +16478,7 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>QUININDÉ</t>
+          <t>SAN LORENZO</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
@@ -16510,7 +16510,7 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>SANTIAGO</t>
+          <t>PALORA</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
@@ -16542,7 +16542,7 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>PALANDA</t>
+          <t>YACUAMBI</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
@@ -16574,7 +16574,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>EL TAMBO</t>
+          <t>DÉLEG</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
@@ -16606,7 +16606,7 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>SAN LORENZO</t>
+          <t>ATACAMES</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
@@ -16638,7 +16638,7 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>DÉLEG</t>
+          <t>SUSCAL</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
@@ -16670,7 +16670,7 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>EL CARMEN</t>
+          <t>PEDERNALES</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
@@ -16702,7 +16702,7 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>PALESTINA</t>
+          <t>PEDRO CARBO</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
@@ -16734,7 +16734,7 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>SUCRE</t>
+          <t>PAJÁN</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">

</xml_diff>